<commit_message>
modified:   __pycache__/dataset.cpython-313.pyc 	new file:   __pycache__/train.cpython-313.pyc 	modified:   dataset.py 	modified:   model_resnet.pt 	new file:   sad_30_scores.xlsx 	new file:   score_images.py 	modified:   test_labels.csv 	new file:   test_metrics_summary.csv 	modified:   test_predictions.csv 	modified:   test_predictions.xlsx 	modified:   test_scores.xlsx 	modified:   train.py 	modified:   train_labels.csv 	modified:   train_scores.xlsx 	new file:   ~$test_predictions.xlsx
</commit_message>
<xml_diff>
--- a/test_scores.xlsx
+++ b/test_scores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G223"/>
+  <dimension ref="A1:G211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2283,70 +2283,70 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a88.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s74.png</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>a88.jpeg</t>
+          <t>s74.png</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D65" t="n">
         <v>0.05</v>
       </c>
       <c r="E65" t="n">
-        <v>0.1</v>
+        <v>0.82</v>
       </c>
       <c r="F65" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s74.png</t>
+          <t>c:\ML_Project\test\Happy\h16.jpg</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>s74.png</t>
+          <t>h16.jpg</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E66" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F66" t="n">
         <v>0.05</v>
       </c>
       <c r="G66" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h16.jpg</t>
+          <t>c:\ML_Project\test\Happy\h70.jpg</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>h16.jpg</t>
+          <t>h70.jpg</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2370,12 +2370,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h70.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h45.jpg</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>h70.jpg</t>
+          <t>new_h45.jpg</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2399,12 +2399,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h45.jpg</t>
+          <t>c:\ML_Project\test\Happy\h30.jpg</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>new_h45.jpg</t>
+          <t>h30.jpg</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2428,70 +2428,70 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h30.jpg</t>
+          <t>c:\ML_Project\test\Fear\f78.jpg</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>h30.jpg</t>
+          <t>f78.jpg</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E70" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F70" t="n">
         <v>0.05</v>
       </c>
       <c r="G70" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f78.jpg</t>
+          <t>c:\ML_Project\test\Angry\a55.jpeg</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>f78.jpg</t>
+          <t>a55.jpeg</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D71" t="n">
         <v>0.05</v>
       </c>
       <c r="E71" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F71" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G71" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a55.jpeg</t>
+          <t>c:\ML_Project\test\Angry\new_a46.jpeg</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>a55.jpeg</t>
+          <t>new_a46.jpeg</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2515,70 +2515,70 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\new_a46.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f9.jpg</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>new_a46.jpeg</t>
+          <t>f9.jpg</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D73" t="n">
         <v>0.05</v>
       </c>
       <c r="E73" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F73" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G73" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f9.jpg</t>
+          <t>c:\ML_Project\test\Sad\s76.jpeg</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>f9.jpg</t>
+          <t>s76.jpeg</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D74" t="n">
         <v>0.05</v>
       </c>
       <c r="E74" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F74" t="n">
         <v>0.05</v>
       </c>
       <c r="G74" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h43.jpg</t>
+          <t>c:\ML_Project\test\Happy\h6.jpg</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>h43.jpg</t>
+          <t>h6.jpg</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2602,12 +2602,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s76.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s97.jpeg</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>s76.jpeg</t>
+          <t>s97.jpeg</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2631,99 +2631,99 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h6.jpg</t>
+          <t>c:\ML_Project\test\Sad\s71.jpeg</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>h6.jpg</t>
+          <t>s71.jpeg</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E77" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F77" t="n">
         <v>0.05</v>
       </c>
       <c r="G77" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s97.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f17.jpg</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>s97.jpeg</t>
+          <t>f17.jpg</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>0.05</v>
       </c>
       <c r="E78" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F78" t="n">
         <v>0.05</v>
       </c>
       <c r="G78" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s71.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h92.jpeg</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>s71.jpeg</t>
+          <t>h92.jpeg</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E79" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F79" t="n">
         <v>0.05</v>
       </c>
       <c r="G79" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f17.jpg</t>
+          <t>c:\ML_Project\test\Fear\f24.jpg</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>f17.jpg</t>
+          <t>f24.jpg</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2747,157 +2747,157 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h92.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s36.jpg</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>h92.jpeg</t>
+          <t>s36.jpg</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E81" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F81" t="n">
         <v>0.05</v>
       </c>
       <c r="G81" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f24.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h50.jpg</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>f24.jpg</t>
+          <t>new_h50.jpg</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E82" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F82" t="n">
         <v>0.05</v>
       </c>
       <c r="G82" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s36.jpg</t>
+          <t>c:\ML_Project\test\Fear\f92.jpeg</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>s36.jpg</t>
+          <t>f92.jpeg</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>0.05</v>
       </c>
       <c r="E83" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F83" t="n">
         <v>0.05</v>
       </c>
       <c r="G83" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h50.jpg</t>
+          <t>c:\ML_Project\test\Fear\f117.jpeg</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>new_h50.jpg</t>
+          <t>f117.jpeg</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E84" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F84" t="n">
         <v>0.05</v>
       </c>
       <c r="G84" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f92.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s8.jpg</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>f92.jpeg</t>
+          <t>s8.jpg</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>0.05</v>
       </c>
       <c r="E85" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F85" t="n">
         <v>0.05</v>
       </c>
       <c r="G85" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f117.jpeg</t>
+          <t>c:\ML_Project\test\Fear\new_f2.png</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>f117.jpeg</t>
+          <t>new_f2.png</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2921,12 +2921,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s8.jpg</t>
+          <t>c:\ML_Project\test\Sad\s53.jpeg</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>s8.jpg</t>
+          <t>s53.jpeg</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2950,99 +2950,99 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f2.png</t>
+          <t>c:\ML_Project\test\Sad\new_s46.jpeg</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>new_f2.png</t>
+          <t>new_s46.jpeg</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>0.05</v>
       </c>
       <c r="E88" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F88" t="n">
         <v>0.05</v>
       </c>
       <c r="G88" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s53.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a84.jpeg</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>s53.jpeg</t>
+          <t>a84.jpeg</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>0.05</v>
       </c>
       <c r="E89" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F89" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G89" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s46.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f99.jpeg</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>new_s46.jpeg</t>
+          <t>f99.jpeg</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>0.05</v>
       </c>
       <c r="E90" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F90" t="n">
         <v>0.05</v>
       </c>
       <c r="G90" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a84.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a43.jpg</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>a84.jpeg</t>
+          <t>a43.jpg</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3066,12 +3066,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f99.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f33.jpg</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>f99.jpeg</t>
+          <t>f33.jpg</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3095,128 +3095,128 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a43.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h17.jpg</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>a43.jpg</t>
+          <t>new_h17.jpg</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E93" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F93" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G93" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f33.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h34.jpg</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>f33.jpg</t>
+          <t>new_h34.jpg</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E94" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F94" t="n">
         <v>0.05</v>
       </c>
       <c r="G94" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h17.jpg</t>
+          <t>c:\ML_Project\test\Sad\new_s11.jpg</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>new_h17.jpg</t>
+          <t>new_s11.jpg</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E95" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F95" t="n">
         <v>0.05</v>
       </c>
       <c r="G95" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h34.jpg</t>
+          <t>c:\ML_Project\test\Sad\s36.jpeg</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>new_h34.jpg</t>
+          <t>s36.jpeg</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E96" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F96" t="n">
         <v>0.05</v>
       </c>
       <c r="G96" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s11.jpg</t>
+          <t>c:\ML_Project\test\Sad\s25.jpg</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>new_s11.jpg</t>
+          <t>s25.jpg</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3240,186 +3240,186 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s36.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a110.jpeg</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>s36.jpeg</t>
+          <t>a110.jpeg</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>0.05</v>
       </c>
       <c r="E98" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F98" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G98" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s25.jpg</t>
+          <t>c:\ML_Project\test\Angry\a56.jpeg</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>s25.jpg</t>
+          <t>a56.jpeg</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>0.05</v>
       </c>
       <c r="E99" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F99" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G99" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a110.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f64.jpg</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>a110.jpeg</t>
+          <t>f64.jpg</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>0.05</v>
       </c>
       <c r="E100" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F100" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G100" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a56.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f15.jpg</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>a56.jpeg</t>
+          <t>f15.jpg</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>0.05</v>
       </c>
       <c r="E101" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F101" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G101" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h25.jpg</t>
+          <t>c:\ML_Project\test\Fear\f17.jpeg</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>h25.jpg</t>
+          <t>f17.jpeg</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E102" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F102" t="n">
         <v>0.05</v>
       </c>
       <c r="G102" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f64.jpg</t>
+          <t>c:\ML_Project\test\Happy\h53.jpg</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>f64.jpg</t>
+          <t>h53.jpg</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E103" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F103" t="n">
         <v>0.05</v>
       </c>
       <c r="G103" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f15.jpg</t>
+          <t>c:\ML_Project\test\Fear\f3.jpg</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>f15.jpg</t>
+          <t>f3.jpg</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3443,41 +3443,41 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f17.jpeg</t>
+          <t>c:\ML_Project\test\Angry\new_a22.jpeg</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>f17.jpeg</t>
+          <t>new_a22.jpeg</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>0.05</v>
       </c>
       <c r="E105" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F105" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G105" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h53.jpg</t>
+          <t>c:\ML_Project\test\Happy\h83.jpeg</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>h53.jpg</t>
+          <t>h83.jpeg</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3501,41 +3501,41 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f3.jpg</t>
+          <t>c:\ML_Project\test\Happy\h56.jpg</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>f3.jpg</t>
+          <t>h56.jpg</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E107" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F107" t="n">
         <v>0.05</v>
       </c>
       <c r="G107" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\new_a22.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a80.jpeg</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>new_a22.jpeg</t>
+          <t>a80.jpeg</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3559,70 +3559,70 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h83.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s19.jpg</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>h83.jpeg</t>
+          <t>s19.jpg</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E109" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F109" t="n">
         <v>0.05</v>
       </c>
       <c r="G109" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h56.jpg</t>
+          <t>c:\ML_Project\test\Sad\s80.jpeg</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>h56.jpg</t>
+          <t>s80.jpeg</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E110" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F110" t="n">
         <v>0.05</v>
       </c>
       <c r="G110" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a80.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a117.jpeg</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>a80.jpeg</t>
+          <t>a117.jpeg</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3646,128 +3646,128 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s19.jpg</t>
+          <t>c:\ML_Project\test\Happy\h17.jpg</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>s19.jpg</t>
+          <t>h17.jpg</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E112" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F112" t="n">
         <v>0.05</v>
       </c>
       <c r="G112" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s80.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h9.jpg</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>s80.jpeg</t>
+          <t>h9.jpg</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E113" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F113" t="n">
         <v>0.05</v>
       </c>
       <c r="G113" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a117.jpeg</t>
+          <t>c:\ML_Project\test\Fear\new_f13.jpeg</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>a117.jpeg</t>
+          <t>new_f13.jpeg</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D114" t="n">
         <v>0.05</v>
       </c>
       <c r="E114" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F114" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G114" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h17.jpg</t>
+          <t>c:\ML_Project\test\Fear\f41.jpg</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>h17.jpg</t>
+          <t>f41.jpg</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E115" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F115" t="n">
         <v>0.05</v>
       </c>
       <c r="G115" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h9.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h6.jpg</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>h9.jpg</t>
+          <t>new_h6.jpg</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3791,128 +3791,128 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f13.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a7.jpg</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>new_f13.jpeg</t>
+          <t>a7.jpg</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D117" t="n">
         <v>0.05</v>
       </c>
       <c r="E117" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F117" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G117" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f41.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h3.jpg</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>f41.jpg</t>
+          <t>new_h3.jpg</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E118" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F118" t="n">
         <v>0.05</v>
       </c>
       <c r="G118" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h6.jpg</t>
+          <t>c:\ML_Project\test\Sad\s38.jpeg</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>new_h6.jpg</t>
+          <t>s38.jpeg</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E119" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F119" t="n">
         <v>0.05</v>
       </c>
       <c r="G119" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a7.jpg</t>
+          <t>c:\ML_Project\test\Happy\h57.jpg</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>a7.jpg</t>
+          <t>h57.jpg</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E120" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F120" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G120" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h3.jpg</t>
+          <t>c:\ML_Project\test\Happy\h84.jpeg</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>new_h3.jpg</t>
+          <t>h84.jpeg</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3936,186 +3936,186 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s38.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f34.jpg</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>s38.jpeg</t>
+          <t>f34.jpg</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D122" t="n">
         <v>0.05</v>
       </c>
       <c r="E122" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F122" t="n">
         <v>0.05</v>
       </c>
       <c r="G122" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h57.jpg</t>
+          <t>c:\ML_Project\test\Angry\a48.jpeg</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>h57.jpg</t>
+          <t>a48.jpeg</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E123" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F123" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G123" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h84.jpeg</t>
+          <t>c:\ML_Project\test\Sad\new_s17.jpg</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>h84.jpeg</t>
+          <t>new_s17.jpg</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E124" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F124" t="n">
         <v>0.05</v>
       </c>
       <c r="G124" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f34.jpg</t>
+          <t>c:\ML_Project\test\Sad\s5.jpg</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>f34.jpg</t>
+          <t>s5.jpg</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D125" t="n">
         <v>0.05</v>
       </c>
       <c r="E125" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F125" t="n">
         <v>0.05</v>
       </c>
       <c r="G125" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a48.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f45.jpg</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>a48.jpeg</t>
+          <t>f45.jpg</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D126" t="n">
         <v>0.05</v>
       </c>
       <c r="E126" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F126" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G126" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s17.jpg</t>
+          <t>c:\ML_Project\test\Fear\new_f40.jpeg</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>new_s17.jpg</t>
+          <t>new_f40.jpeg</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D127" t="n">
         <v>0.05</v>
       </c>
       <c r="E127" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F127" t="n">
         <v>0.05</v>
       </c>
       <c r="G127" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s5.jpg</t>
+          <t>c:\ML_Project\test\Sad\new_s15.jpg</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>s5.jpg</t>
+          <t>new_s15.jpg</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -4139,12 +4139,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f45.jpg</t>
+          <t>c:\ML_Project\test\Fear\f88.jpeg</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>f45.jpg</t>
+          <t>f88.jpeg</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -4168,41 +4168,41 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a83.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f58.jpeg</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>a83.jpeg</t>
+          <t>f58.jpeg</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D130" t="n">
         <v>0.05</v>
       </c>
       <c r="E130" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F130" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G130" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f40.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f105.jpeg</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>new_f40.jpeg</t>
+          <t>f105.jpeg</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -4226,41 +4226,41 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s15.jpg</t>
+          <t>c:\ML_Project\test\Angry\a111.jpeg</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>new_s15.jpg</t>
+          <t>a111.jpeg</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D132" t="n">
         <v>0.05</v>
       </c>
       <c r="E132" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F132" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G132" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f88.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f14.jpeg</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>f88.jpeg</t>
+          <t>f14.jpeg</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4284,302 +4284,302 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f58.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a69.jpg</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>f58.jpeg</t>
+          <t>a69.jpg</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D134" t="n">
         <v>0.05</v>
       </c>
       <c r="E134" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F134" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G134" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f105.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h5.jpg</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>f105.jpeg</t>
+          <t>h5.jpg</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E135" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F135" t="n">
         <v>0.05</v>
       </c>
       <c r="G135" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a111.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h20.jpg</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>a111.jpeg</t>
+          <t>h20.jpg</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E136" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F136" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G136" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f14.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s34.webp</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>f14.jpeg</t>
+          <t>s34.webp</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D137" t="n">
         <v>0.05</v>
       </c>
       <c r="E137" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F137" t="n">
         <v>0.05</v>
       </c>
       <c r="G137" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a69.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h39.jpg</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>a69.jpg</t>
+          <t>new_h39.jpg</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E138" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F138" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G138" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h5.jpg</t>
+          <t>c:\ML_Project\test\Fear\new_f50.jpeg</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>h5.jpg</t>
+          <t>new_f50.jpeg</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E139" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F139" t="n">
         <v>0.05</v>
       </c>
       <c r="G139" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h20.jpg</t>
+          <t>c:\ML_Project\test\Fear\f101.jpeg</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>h20.jpg</t>
+          <t>f101.jpeg</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E140" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F140" t="n">
         <v>0.05</v>
       </c>
       <c r="G140" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s34.webp</t>
+          <t>c:\ML_Project\test\Happy\new_h49.jpg</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>s34.webp</t>
+          <t>new_h49.jpg</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E141" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F141" t="n">
         <v>0.05</v>
       </c>
       <c r="G141" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h39.jpg</t>
+          <t>c:\ML_Project\test\Angry\a6.jpg</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>new_h39.jpg</t>
+          <t>a6.jpg</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E142" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F142" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G142" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f50.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s55.jpeg</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>new_f50.jpeg</t>
+          <t>s55.jpeg</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D143" t="n">
         <v>0.05</v>
       </c>
       <c r="E143" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F143" t="n">
         <v>0.05</v>
       </c>
       <c r="G143" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f101.jpeg</t>
+          <t>c:\ML_Project\test\Fear\new_f53.jpeg</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>f101.jpeg</t>
+          <t>new_f53.jpeg</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -4603,12 +4603,12 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f77.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f118.webp</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>f77.jpeg</t>
+          <t>f118.webp</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -4632,215 +4632,215 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h49.jpg</t>
+          <t>c:\ML_Project\test\Fear\f47.jpg</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>new_h49.jpg</t>
+          <t>f47.jpg</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E146" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F146" t="n">
         <v>0.05</v>
       </c>
       <c r="G146" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a6.jpg</t>
+          <t>c:\ML_Project\test\Sad\new_download (6).jpeg</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>a6.jpg</t>
+          <t>new_download (6).jpeg</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D147" t="n">
         <v>0.05</v>
       </c>
       <c r="E147" t="n">
-        <v>0.1</v>
+        <v>0.82</v>
       </c>
       <c r="F147" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G147" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s55.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a99.jpeg</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>s55.jpeg</t>
+          <t>a99.jpeg</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D148" t="n">
         <v>0.05</v>
       </c>
       <c r="E148" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F148" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G148" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f45.jpg</t>
+          <t>c:\ML_Project\test\Angry\a98.jpeg</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>f45.jpg</t>
+          <t>a98.jpeg</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D149" t="n">
         <v>0.05</v>
       </c>
       <c r="E149" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F149" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G149" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f53.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h2.jpg</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>new_f53.jpeg</t>
+          <t>h2.jpg</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E150" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F150" t="n">
         <v>0.05</v>
       </c>
       <c r="G150" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f118.webp</t>
+          <t>c:\ML_Project\test\Angry\a70.jpeg</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>f118.webp</t>
+          <t>a70.jpeg</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D151" t="n">
         <v>0.05</v>
       </c>
       <c r="E151" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F151" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G151" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f47.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_h24.jpg</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>f47.jpg</t>
+          <t>new_h24.jpg</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E152" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F152" t="n">
         <v>0.05</v>
       </c>
       <c r="G152" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_download (6).jpeg</t>
+          <t>c:\ML_Project\test\Sad\s9.jpg</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>new_download (6).jpeg</t>
+          <t>s9.jpg</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -4864,12 +4864,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a99.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a118.jpeg</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>a99.jpeg</t>
+          <t>a118.jpeg</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4893,12 +4893,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a98.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a47.jpg</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>a98.jpeg</t>
+          <t>a47.jpg</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -4922,70 +4922,70 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h2.jpg</t>
+          <t>c:\ML_Project\test\Fear\f57.jpg</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>h2.jpg</t>
+          <t>f57.jpg</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E156" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F156" t="n">
         <v>0.05</v>
       </c>
       <c r="G156" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a70.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f15.jpeg</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>a70.jpeg</t>
+          <t>f15.jpeg</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D157" t="n">
         <v>0.05</v>
       </c>
       <c r="E157" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F157" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G157" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h24.jpg</t>
+          <t>c:\ML_Project\test\Happy\h14.jpg</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>new_h24.jpg</t>
+          <t>h14.jpg</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -5009,215 +5009,215 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s9.jpg</t>
+          <t>c:\ML_Project\test\Angry\new_a10.jpeg</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>s9.jpg</t>
+          <t>new_a10.jpeg</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D159" t="n">
         <v>0.05</v>
       </c>
       <c r="E159" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F159" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G159" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a118.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s46.jpeg</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>a118.jpeg</t>
+          <t>s46.jpeg</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D160" t="n">
         <v>0.05</v>
       </c>
       <c r="E160" t="n">
-        <v>0.1</v>
+        <v>0.82</v>
       </c>
       <c r="F160" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G160" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a47.jpg</t>
+          <t>c:\ML_Project\test\Happy\h98.jpeg</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>a47.jpg</t>
+          <t>h98.jpeg</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E161" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F161" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G161" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f57.jpg</t>
+          <t>c:\ML_Project\test\Happy\h99.jpeg</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>f57.jpg</t>
+          <t>h99.jpeg</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E162" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="F162" t="n">
         <v>0.05</v>
       </c>
       <c r="G162" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f2.jpg</t>
+          <t>c:\ML_Project\test\Sad\s89.jpeg</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>f2.jpg</t>
+          <t>s89.jpeg</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D163" t="n">
         <v>0.05</v>
       </c>
       <c r="E163" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F163" t="n">
         <v>0.05</v>
       </c>
       <c r="G163" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f15.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s55.jpg</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>f15.jpeg</t>
+          <t>s55.jpg</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D164" t="n">
         <v>0.05</v>
       </c>
       <c r="E164" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F164" t="n">
         <v>0.05</v>
       </c>
       <c r="G164" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h14.jpg</t>
+          <t>c:\ML_Project\test\Fear\new_f1.jpeg</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>h14.jpg</t>
+          <t>new_f1.jpeg</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E165" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F165" t="n">
         <v>0.05</v>
       </c>
       <c r="G165" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\new_a10.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a42.jpg</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>new_a10.jpeg</t>
+          <t>a42.jpg</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -5241,128 +5241,128 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h84.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f5.jpg</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>h84.jpeg</t>
+          <t>f5.jpg</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E167" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F167" t="n">
         <v>0.05</v>
       </c>
       <c r="G167" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s46.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a78.jpg</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>s46.jpeg</t>
+          <t>a78.jpg</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D168" t="n">
         <v>0.05</v>
       </c>
       <c r="E168" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F168" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G168" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h98.jpeg</t>
+          <t>c:\ML_Project\test\Fear\new_f36.jpeg</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>h98.jpeg</t>
+          <t>new_f36.jpeg</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E169" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F169" t="n">
         <v>0.05</v>
       </c>
       <c r="G169" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h14.jpg</t>
+          <t>c:\ML_Project\test\Fear\f51.jpg</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>h14.jpg</t>
+          <t>f51.jpg</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E170" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="F170" t="n">
         <v>0.05</v>
       </c>
       <c r="G170" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h99.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h68.jpg</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>h99.jpeg</t>
+          <t>h68.jpg</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s89.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s79.jpeg</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>s89.jpeg</t>
+          <t>s79.jpeg</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -5415,41 +5415,41 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s55.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_images (54).jpg</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>s55.jpg</t>
+          <t>new_images (54).jpg</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E173" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F173" t="n">
         <v>0.05</v>
       </c>
       <c r="G173" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f1.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f36.jpg</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>new_f1.jpeg</t>
+          <t>f36.jpg</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5473,12 +5473,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a42.jpg</t>
+          <t>c:\ML_Project\test\Angry\new_a51.jpeg</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>a42.jpg</t>
+          <t>new_a51.jpeg</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -5502,70 +5502,70 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f5.jpg</t>
+          <t>c:\ML_Project\test\Sad\new_klk.jpeg</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>f5.jpg</t>
+          <t>new_klk.jpeg</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D176" t="n">
         <v>0.05</v>
       </c>
       <c r="E176" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F176" t="n">
         <v>0.05</v>
       </c>
       <c r="G176" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a78.jpg</t>
+          <t>c:\ML_Project\test\Happy\new_images (47).jpg</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>a78.jpg</t>
+          <t>new_images (47).jpg</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E177" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="F177" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G177" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_f36.jpeg</t>
+          <t>c:\ML_Project\test\Fear\f46.jpg</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>new_f36.jpeg</t>
+          <t>f46.jpg</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -5589,128 +5589,128 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f51.jpg</t>
+          <t>c:\ML_Project\test\Angry\a87.jpeg</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>f51.jpg</t>
+          <t>a87.jpeg</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D179" t="n">
         <v>0.05</v>
       </c>
       <c r="E179" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F179" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G179" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h68.jpg</t>
+          <t>c:\ML_Project\test\Sad\s110.jpeg</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>h68.jpg</t>
+          <t>s110.jpeg</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E180" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F180" t="n">
         <v>0.05</v>
       </c>
       <c r="G180" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s79.jpeg</t>
+          <t>c:\ML_Project\test\Happy\new_h47.jpg</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>s79.jpeg</t>
+          <t>new_h47.jpg</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E181" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F181" t="n">
         <v>0.05</v>
       </c>
       <c r="G181" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_images (54).jpg</t>
+          <t>c:\ML_Project\test\Sad\new_s48.jpeg</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>new_images (54).jpg</t>
+          <t>new_s48.jpeg</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E182" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F182" t="n">
         <v>0.05</v>
       </c>
       <c r="G182" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f36.jpg</t>
+          <t>c:\ML_Project\test\Fear\new_images (1).jpeg</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>f36.jpg</t>
+          <t>new_images (1).jpeg</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -5734,12 +5734,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\new_a51.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a22.jpg</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>new_a51.jpeg</t>
+          <t>a22.jpg</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -5763,12 +5763,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_klk.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s103.jpeg</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>new_klk.jpeg</t>
+          <t>s103.jpeg</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -5792,41 +5792,41 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_images (47).jpg</t>
+          <t>c:\ML_Project\test\Sad\s84.jpeg</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>new_images (47).jpg</t>
+          <t>s84.jpeg</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E186" t="n">
-        <v>0.05</v>
+        <v>0.82</v>
       </c>
       <c r="F186" t="n">
         <v>0.05</v>
       </c>
       <c r="G186" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s32.jpg</t>
+          <t>c:\ML_Project\test\Sad\s81.jpeg</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>s32.jpg</t>
+          <t>s81.jpeg</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5850,41 +5850,41 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\f46.jpg</t>
+          <t>c:\ML_Project\test\Sad\s77.jpeg</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>f46.jpg</t>
+          <t>s77.jpeg</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D188" t="n">
         <v>0.05</v>
       </c>
       <c r="E188" t="n">
-        <v>0.15</v>
+        <v>0.82</v>
       </c>
       <c r="F188" t="n">
         <v>0.05</v>
       </c>
       <c r="G188" t="n">
-        <v>0.75</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a87.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a26.jpg</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>a87.jpeg</t>
+          <t>a26.jpg</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5908,41 +5908,41 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a7.jpg</t>
+          <t>c:\ML_Project\test\Sad\s50.jpg</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>a7.jpg</t>
+          <t>s50.jpg</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D190" t="n">
         <v>0.05</v>
       </c>
       <c r="E190" t="n">
-        <v>0.1</v>
+        <v>0.82</v>
       </c>
       <c r="F190" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G190" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s110.jpeg</t>
+          <t>c:\ML_Project\test\Sad\new_s50.jpeg</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>s110.jpeg</t>
+          <t>new_s50.jpeg</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -5966,128 +5966,128 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h47.jpg</t>
+          <t>c:\ML_Project\test\Angry\a23.jpg</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>new_h47.jpg</t>
+          <t>a23.jpg</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E192" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F192" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G192" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s48.jpeg</t>
+          <t>c:\ML_Project\test\Happy\new_h29.jpg</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>new_s48.jpeg</t>
+          <t>new_h29.jpg</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E193" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F193" t="n">
         <v>0.05</v>
       </c>
       <c r="G193" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Fear\new_images (1).jpeg</t>
+          <t>c:\ML_Project\test\Angry\new_a38.jpeg</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>new_images (1).jpeg</t>
+          <t>new_a38.jpeg</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Fear</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D194" t="n">
         <v>0.05</v>
       </c>
       <c r="E194" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F194" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G194" t="n">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a22.jpg</t>
+          <t>c:\ML_Project\test\Sad\s83.jpeg</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>a22.jpg</t>
+          <t>s83.jpeg</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Sad</t>
         </is>
       </c>
       <c r="D195" t="n">
         <v>0.05</v>
       </c>
       <c r="E195" t="n">
-        <v>0.1</v>
+        <v>0.82</v>
       </c>
       <c r="F195" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G195" t="n">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s103.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s10.jpg</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>s103.jpeg</t>
+          <t>s10.jpg</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -6111,41 +6111,41 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\h83.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a79.jpg</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>h83.jpeg</t>
+          <t>a79.jpg</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Happy</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>0.85</v>
+        <v>0.05</v>
       </c>
       <c r="E197" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="F197" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G197" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s84.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s115.jpeg</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>s84.jpeg</t>
+          <t>s115.jpeg</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -6169,12 +6169,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s81.jpeg</t>
+          <t>c:\ML_Project\test\Sad\s33.jpg</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>s81.jpeg</t>
+          <t>s33.jpg</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -6198,99 +6198,99 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s77.jpeg</t>
+          <t>c:\ML_Project\test\Happy\h26.jpg</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>s77.jpeg</t>
+          <t>h26.jpg</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>0.05</v>
+        <v>0.85</v>
       </c>
       <c r="E200" t="n">
-        <v>0.82</v>
+        <v>0.05</v>
       </c>
       <c r="F200" t="n">
         <v>0.05</v>
       </c>
       <c r="G200" t="n">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a26.jpg</t>
+          <t>c:\ML_Project\test\Fear\new_f30.jpeg</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>a26.jpg</t>
+          <t>new_f30.jpeg</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Angry</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D201" t="n">
         <v>0.05</v>
       </c>
       <c r="E201" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F201" t="n">
-        <v>0.75</v>
+        <v>0.05</v>
       </c>
       <c r="G201" t="n">
-        <v>0.1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s50.jpg</t>
+          <t>c:\ML_Project\test\Fear\f31.jpg</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>s50.jpg</t>
+          <t>f31.jpg</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Fear</t>
         </is>
       </c>
       <c r="D202" t="n">
         <v>0.05</v>
       </c>
       <c r="E202" t="n">
-        <v>0.82</v>
+        <v>0.15</v>
       </c>
       <c r="F202" t="n">
         <v>0.05</v>
       </c>
       <c r="G202" t="n">
-        <v>0.08</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\new_s50.jpeg</t>
+          <t>c:\ML_Project\test\Sad\new_s6.jpg</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>new_s50.jpeg</t>
+          <t>new_s6.jpg</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -6314,12 +6314,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a23.jpg</t>
+          <t>c:\ML_Project\test\Angry\a37.jpg</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>a23.jpg</t>
+          <t>a37.jpg</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -6343,12 +6343,12 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Happy\new_h29.jpg</t>
+          <t>c:\ML_Project\test\Happy\h91.jpeg</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>new_h29.jpg</t>
+          <t>h91.jpeg</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -6372,12 +6372,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\new_a38.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a71.jpeg</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>new_a38.jpeg</t>
+          <t>a71.jpeg</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -6401,70 +6401,70 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s83.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a50.jpg</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>s83.jpeg</t>
+          <t>a50.jpg</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D207" t="n">
         <v>0.05</v>
       </c>
       <c r="E207" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F207" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G207" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s10.jpg</t>
+          <t>c:\ML_Project\test\Angry\a51.jpg</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>s10.jpg</t>
+          <t>a51.jpg</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D208" t="n">
         <v>0.05</v>
       </c>
       <c r="E208" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F208" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G208" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Angry\a79.jpg</t>
+          <t>c:\ML_Project\test\Angry\a100.jpeg</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>a79.jpg</t>
+          <t>a100.jpeg</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -6488,41 +6488,41 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s115.jpeg</t>
+          <t>c:\ML_Project\test\Angry\a94.webp</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>s115.jpeg</t>
+          <t>a94.webp</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Angry</t>
         </is>
       </c>
       <c r="D210" t="n">
         <v>0.05</v>
       </c>
       <c r="E210" t="n">
-        <v>0.82</v>
+        <v>0.1</v>
       </c>
       <c r="F210" t="n">
-        <v>0.05</v>
+        <v>0.75</v>
       </c>
       <c r="G210" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>c:\ML_Project\test\Sad\s33.jpg</t>
+          <t>c:\ML_Project\test\Sad\s45.jpeg</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>s33.jpg</t>
+          <t>s45.jpeg</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -6540,354 +6540,6 @@
         <v>0.05</v>
       </c>
       <c r="G211" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Happy\h26.jpg</t>
-        </is>
-      </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>h26.jpg</t>
-        </is>
-      </c>
-      <c r="C212" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="D212" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E212" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F212" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G212" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Fear\new_f30.jpeg</t>
-        </is>
-      </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>new_f30.jpeg</t>
-        </is>
-      </c>
-      <c r="C213" t="inlineStr">
-        <is>
-          <t>Fear</t>
-        </is>
-      </c>
-      <c r="D213" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E213" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F213" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G213" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Fear\f31.jpg</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>f31.jpg</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>Fear</t>
-        </is>
-      </c>
-      <c r="D214" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E214" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F214" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G214" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Sad\new_s6.jpg</t>
-        </is>
-      </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>new_s6.jpg</t>
-        </is>
-      </c>
-      <c r="C215" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="D215" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E215" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F215" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G215" t="n">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a37.jpg</t>
-        </is>
-      </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>a37.jpg</t>
-        </is>
-      </c>
-      <c r="C216" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D216" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E216" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F216" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G216" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Happy\h91.jpeg</t>
-        </is>
-      </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>h91.jpeg</t>
-        </is>
-      </c>
-      <c r="C217" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="D217" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E217" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F217" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G217" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a71.jpeg</t>
-        </is>
-      </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>a71.jpeg</t>
-        </is>
-      </c>
-      <c r="C218" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D218" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E218" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F218" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G218" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a50.jpg</t>
-        </is>
-      </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>a50.jpg</t>
-        </is>
-      </c>
-      <c r="C219" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D219" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E219" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F219" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G219" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a51.jpg</t>
-        </is>
-      </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>a51.jpg</t>
-        </is>
-      </c>
-      <c r="C220" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D220" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E220" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F220" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G220" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a100.jpeg</t>
-        </is>
-      </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>a100.jpeg</t>
-        </is>
-      </c>
-      <c r="C221" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D221" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E221" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F221" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G221" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Angry\a94.webp</t>
-        </is>
-      </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>a94.webp</t>
-        </is>
-      </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Angry</t>
-        </is>
-      </c>
-      <c r="D222" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E222" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F222" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G222" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>c:\ML_Project\test\Sad\s45.jpeg</t>
-        </is>
-      </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>s45.jpeg</t>
-        </is>
-      </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="D223" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="E223" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F223" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G223" t="n">
         <v>0.08</v>
       </c>
     </row>

</xml_diff>